<commit_message>
Added Aliases, initial version
</commit_message>
<xml_diff>
--- a/Docs/poms.xlsx
+++ b/Docs/poms.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28227"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Coding\Ring\RingCsharp\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7564137C-C4B2-455B-8BF7-959A67EFBEC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DF09FC8-A67C-4677-95F4-4E8131B1DDFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" firstSheet="5" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="table" sheetId="1" r:id="rId1"/>
@@ -26,9 +26,10 @@
     <sheet name="sequence" sheetId="12" r:id="rId11"/>
     <sheet name="assembly" sheetId="13" r:id="rId12"/>
     <sheet name="tablespace" sheetId="16" r:id="rId13"/>
-    <sheet name="node" sheetId="9" r:id="rId14"/>
-    <sheet name="partition" sheetId="10" r:id="rId15"/>
-    <sheet name="service" sheetId="11" r:id="rId16"/>
+    <sheet name="alias" sheetId="17" r:id="rId14"/>
+    <sheet name="node" sheetId="9" r:id="rId15"/>
+    <sheet name="partition" sheetId="10" r:id="rId16"/>
+    <sheet name="service" sheetId="11" r:id="rId17"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -48,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="642" uniqueCount="102">
   <si>
     <t xml:space="preserve">id </t>
   </si>
@@ -339,6 +340,21 @@
   </si>
   <si>
     <t>[1,127]</t>
+  </si>
+  <si>
+    <t>table id</t>
+  </si>
+  <si>
+    <t>alias id</t>
+  </si>
+  <si>
+    <t>usual bit + 1 byte for entityType</t>
+  </si>
+  <si>
+    <t>target entity id</t>
+  </si>
+  <si>
+    <t>name of entity</t>
   </si>
 </sst>
 </file>
@@ -1621,6 +1637,177 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BAA8DBA-5A44-4DE5-B13B-8DEA82490ADB}">
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr defaultColWidth="12.68359375" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <cols>
+    <col min="1" max="1" width="12.41796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.83984375" customWidth="1"/>
+    <col min="4" max="4" width="14.26171875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C5">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" t="s">
+        <v>62</v>
+      </c>
+      <c r="C7" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A8" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C8" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A9" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A10" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A11" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B11" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A13" t="s">
+        <v>37</v>
+      </c>
+      <c r="B13" s="4"/>
+      <c r="C13" s="8" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A14" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A16" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B17">
+        <v>1</v>
+      </c>
+      <c r="C17" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>84</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
@@ -1801,7 +1988,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
   <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
@@ -1982,7 +2169,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
   <dimension ref="A1:E14"/>
   <sheetFormatPr defaultColWidth="12.68359375" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>

</xml_diff>

<commit_message>
Moved Constraint to Meta struct: part 2
</commit_message>
<xml_diff>
--- a/Docs/poms.xlsx
+++ b/Docs/poms.xlsx
@@ -1,16 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28227"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4507"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Coding\Ring\RingCsharp\Docs\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DF09FC8-A67C-4677-95F4-4E8131B1DDFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" firstSheet="5" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="-90" windowWidth="23235" windowHeight="12435" activeTab="17"/>
   </bookViews>
   <sheets>
     <sheet name="table" sheetId="1" r:id="rId1"/>
@@ -30,8 +24,9 @@
     <sheet name="node" sheetId="9" r:id="rId15"/>
     <sheet name="partition" sheetId="10" r:id="rId16"/>
     <sheet name="service" sheetId="11" r:id="rId17"/>
+    <sheet name="constraint" sheetId="18" r:id="rId18"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="125725"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -49,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="642" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="688" uniqueCount="106">
   <si>
     <t xml:space="preserve">id </t>
   </si>
@@ -355,13 +350,25 @@
   </si>
   <si>
     <t>name of entity</t>
+  </si>
+  <si>
+    <t>constraint_id</t>
+  </si>
+  <si>
+    <t>constraint_type</t>
+  </si>
+  <si>
+    <t>ck_@meta_001</t>
+  </si>
+  <si>
+    <t>min_value; max_value; column1; column2; ….</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -750,23 +757,23 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E14"/>
-  <sheetFormatPr defaultColWidth="12.68359375" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.83984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.68359375" customWidth="1"/>
-    <col min="4" max="4" width="26.15625" customWidth="1"/>
+    <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.7109375" customWidth="1"/>
+    <col min="4" max="4" width="26.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:5">
       <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
@@ -780,7 +787,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:5">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -794,7 +801,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:5">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -811,7 +818,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:5">
       <c r="A4" s="2" t="s">
         <v>35</v>
       </c>
@@ -828,7 +835,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:5">
       <c r="A5" s="2" t="s">
         <v>16</v>
       </c>
@@ -839,7 +846,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:5">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
@@ -853,7 +860,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:5">
       <c r="A7" s="1" t="s">
         <v>14</v>
       </c>
@@ -867,7 +874,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:5">
       <c r="A8" s="7" t="s">
         <v>1</v>
       </c>
@@ -881,7 +888,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:5">
       <c r="A9" s="1" t="s">
         <v>2</v>
       </c>
@@ -892,7 +899,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:5">
       <c r="A10" s="1" t="s">
         <v>3</v>
       </c>
@@ -903,7 +910,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:5">
       <c r="A11" s="1" t="s">
         <v>42</v>
       </c>
@@ -917,7 +924,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:5">
       <c r="A13" t="s">
         <v>37</v>
       </c>
@@ -926,7 +933,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:5">
       <c r="A14" t="s">
         <v>38</v>
       </c>
@@ -944,16 +951,16 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultColWidth="12.68359375" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="12.41796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.83984375" customWidth="1"/>
-    <col min="4" max="4" width="14.26171875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.85546875" customWidth="1"/>
+    <col min="4" max="4" width="14.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:4">
       <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
@@ -967,7 +974,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:4">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -978,7 +985,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:4">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -989,7 +996,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:4">
       <c r="A4" s="2" t="s">
         <v>35</v>
       </c>
@@ -1000,7 +1007,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:4">
       <c r="A5" s="2" t="s">
         <v>16</v>
       </c>
@@ -1011,7 +1018,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:4">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
@@ -1019,7 +1026,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:4">
       <c r="A7" s="1" t="s">
         <v>14</v>
       </c>
@@ -1027,7 +1034,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:4">
       <c r="A8" s="7" t="s">
         <v>1</v>
       </c>
@@ -1038,7 +1045,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:4">
       <c r="A9" s="1" t="s">
         <v>2</v>
       </c>
@@ -1049,7 +1056,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:4">
       <c r="A10" s="1" t="s">
         <v>3</v>
       </c>
@@ -1057,7 +1064,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:4">
       <c r="A11" s="1" t="s">
         <v>42</v>
       </c>
@@ -1065,7 +1072,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:4">
       <c r="A13" t="s">
         <v>37</v>
       </c>
@@ -1074,7 +1081,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:4">
       <c r="A14" t="s">
         <v>38</v>
       </c>
@@ -1082,12 +1089,12 @@
         <v>45</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:4">
       <c r="A16" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="2:3">
       <c r="B17">
         <v>1</v>
       </c>
@@ -1095,7 +1102,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="2:3">
       <c r="B18">
         <v>2</v>
       </c>
@@ -1109,16 +1116,16 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E14"/>
-  <sheetFormatPr defaultColWidth="12.68359375" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.83984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.68359375" customWidth="1"/>
-    <col min="4" max="4" width="26.15625" customWidth="1"/>
+    <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.7109375" customWidth="1"/>
+    <col min="4" max="4" width="26.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:5">
       <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
@@ -1132,7 +1139,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:5">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -1146,7 +1153,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:5">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -1163,7 +1170,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:5">
       <c r="A4" s="2" t="s">
         <v>35</v>
       </c>
@@ -1180,7 +1187,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:5">
       <c r="A5" s="2" t="s">
         <v>16</v>
       </c>
@@ -1194,7 +1201,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:5">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
@@ -1209,7 +1216,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:5">
       <c r="A7" s="1" t="s">
         <v>14</v>
       </c>
@@ -1218,7 +1225,7 @@
       </c>
       <c r="C7" s="10"/>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:5">
       <c r="A8" s="7" t="s">
         <v>1</v>
       </c>
@@ -1229,7 +1236,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:5">
       <c r="A9" s="1" t="s">
         <v>2</v>
       </c>
@@ -1237,7 +1244,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:5">
       <c r="A10" s="1" t="s">
         <v>3</v>
       </c>
@@ -1248,7 +1255,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:5">
       <c r="A11" s="1" t="s">
         <v>42</v>
       </c>
@@ -1262,7 +1269,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:5">
       <c r="A13" t="s">
         <v>37</v>
       </c>
@@ -1271,7 +1278,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:5">
       <c r="A14" t="s">
         <v>38</v>
       </c>
@@ -1289,16 +1296,16 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E14"/>
-  <sheetFormatPr defaultColWidth="12.68359375" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.83984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.68359375" customWidth="1"/>
-    <col min="4" max="4" width="26.15625" customWidth="1"/>
+    <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.7109375" customWidth="1"/>
+    <col min="4" max="4" width="26.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:5">
       <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
@@ -1312,7 +1319,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:5">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -1326,7 +1333,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:5">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -1343,7 +1350,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:5">
       <c r="A4" s="2" t="s">
         <v>35</v>
       </c>
@@ -1360,7 +1367,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:5">
       <c r="A5" s="2" t="s">
         <v>16</v>
       </c>
@@ -1374,7 +1381,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:5">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
@@ -1389,7 +1396,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:5">
       <c r="A7" s="1" t="s">
         <v>14</v>
       </c>
@@ -1398,7 +1405,7 @@
       </c>
       <c r="C7" s="10"/>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:5">
       <c r="A8" s="7" t="s">
         <v>1</v>
       </c>
@@ -1409,7 +1416,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:5">
       <c r="A9" s="1" t="s">
         <v>2</v>
       </c>
@@ -1417,7 +1424,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:5">
       <c r="A10" s="1" t="s">
         <v>3</v>
       </c>
@@ -1428,7 +1435,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:5">
       <c r="A11" s="1" t="s">
         <v>42</v>
       </c>
@@ -1442,7 +1449,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:5">
       <c r="A13" t="s">
         <v>37</v>
       </c>
@@ -1451,7 +1458,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:5">
       <c r="A14" t="s">
         <v>38</v>
       </c>
@@ -1466,16 +1473,16 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultColWidth="12.68359375" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="12.41796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.83984375" customWidth="1"/>
-    <col min="4" max="4" width="14.26171875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.85546875" customWidth="1"/>
+    <col min="4" max="4" width="14.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:4">
       <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
@@ -1489,7 +1496,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:4">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -1500,7 +1507,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:4">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -1511,7 +1518,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:4">
       <c r="A4" s="2" t="s">
         <v>35</v>
       </c>
@@ -1522,7 +1529,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:4">
       <c r="A5" s="2" t="s">
         <v>16</v>
       </c>
@@ -1533,7 +1540,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:4">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
@@ -1544,7 +1551,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:4">
       <c r="A7" s="1" t="s">
         <v>14</v>
       </c>
@@ -1555,7 +1562,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:4">
       <c r="A8" s="7" t="s">
         <v>1</v>
       </c>
@@ -1566,7 +1573,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:4">
       <c r="A9" s="1" t="s">
         <v>2</v>
       </c>
@@ -1574,7 +1581,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:4">
       <c r="A10" s="1" t="s">
         <v>3</v>
       </c>
@@ -1585,7 +1592,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:4">
       <c r="A11" s="1" t="s">
         <v>42</v>
       </c>
@@ -1593,7 +1600,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:4">
       <c r="A13" t="s">
         <v>37</v>
       </c>
@@ -1602,7 +1609,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:4">
       <c r="A14" t="s">
         <v>38</v>
       </c>
@@ -1610,12 +1617,12 @@
         <v>45</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:4">
       <c r="A16" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="2:3">
       <c r="B17">
         <v>1</v>
       </c>
@@ -1623,7 +1630,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="2:3">
       <c r="B18">
         <v>2</v>
       </c>
@@ -1637,16 +1644,16 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BAA8DBA-5A44-4DE5-B13B-8DEA82490ADB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultColWidth="12.68359375" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="12.41796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.83984375" customWidth="1"/>
-    <col min="4" max="4" width="14.26171875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.85546875" customWidth="1"/>
+    <col min="4" max="4" width="14.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:4">
       <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
@@ -1660,7 +1667,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:4">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -1671,7 +1678,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:4">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -1682,7 +1689,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:4">
       <c r="A4" s="2" t="s">
         <v>35</v>
       </c>
@@ -1693,7 +1700,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:4">
       <c r="A5" s="2" t="s">
         <v>16</v>
       </c>
@@ -1704,7 +1711,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:4">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
@@ -1715,7 +1722,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:4">
       <c r="A7" s="1" t="s">
         <v>14</v>
       </c>
@@ -1726,7 +1733,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:4">
       <c r="A8" s="7" t="s">
         <v>1</v>
       </c>
@@ -1737,7 +1744,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:4">
       <c r="A9" s="1" t="s">
         <v>2</v>
       </c>
@@ -1745,7 +1752,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:4">
       <c r="A10" s="1" t="s">
         <v>3</v>
       </c>
@@ -1756,7 +1763,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:4">
       <c r="A11" s="1" t="s">
         <v>42</v>
       </c>
@@ -1764,7 +1771,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:4">
       <c r="A13" t="s">
         <v>37</v>
       </c>
@@ -1773,7 +1780,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:4">
       <c r="A14" t="s">
         <v>38</v>
       </c>
@@ -1781,12 +1788,12 @@
         <v>45</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:4">
       <c r="A16" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="2:3">
       <c r="B17">
         <v>1</v>
       </c>
@@ -1794,7 +1801,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="2:3">
       <c r="B18">
         <v>2</v>
       </c>
@@ -1808,17 +1815,17 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.83984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.68359375" customWidth="1"/>
-    <col min="3" max="3" width="28.68359375" customWidth="1"/>
-    <col min="4" max="4" width="14.26171875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" customWidth="1"/>
+    <col min="3" max="3" width="28.7109375" customWidth="1"/>
+    <col min="4" max="4" width="14.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:4">
       <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
@@ -1832,7 +1839,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:4">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -1846,7 +1853,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:4">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -1860,7 +1867,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:4">
       <c r="A4" s="2" t="s">
         <v>16</v>
       </c>
@@ -1874,7 +1881,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:4">
       <c r="A5" s="1" t="s">
         <v>35</v>
       </c>
@@ -1888,7 +1895,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:4">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
@@ -1902,7 +1909,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:4">
       <c r="A7" s="1" t="s">
         <v>14</v>
       </c>
@@ -1916,7 +1923,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:4">
       <c r="A8" s="7" t="s">
         <v>1</v>
       </c>
@@ -1930,7 +1937,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:4">
       <c r="A9" s="1" t="s">
         <v>2</v>
       </c>
@@ -1938,7 +1945,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:4">
       <c r="A10" s="1" t="s">
         <v>3</v>
       </c>
@@ -1949,7 +1956,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:4">
       <c r="A11" s="1" t="s">
         <v>42</v>
       </c>
@@ -1963,7 +1970,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:4">
       <c r="A13" t="s">
         <v>37</v>
       </c>
@@ -1972,7 +1979,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:4">
       <c r="A14" t="s">
         <v>38</v>
       </c>
@@ -1982,24 +1989,24 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C10" r:id="rId1" xr:uid="{00000000-0004-0000-0D00-000000000000}"/>
+    <hyperlink ref="C10" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.83984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.68359375" customWidth="1"/>
-    <col min="3" max="3" width="28.68359375" customWidth="1"/>
-    <col min="4" max="4" width="14.26171875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" customWidth="1"/>
+    <col min="3" max="3" width="28.7109375" customWidth="1"/>
+    <col min="4" max="4" width="14.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:4">
       <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
@@ -2013,7 +2020,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:4">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -2027,7 +2034,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:4">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -2041,7 +2048,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:4">
       <c r="A4" s="2" t="s">
         <v>16</v>
       </c>
@@ -2055,7 +2062,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:4">
       <c r="A5" s="1" t="s">
         <v>35</v>
       </c>
@@ -2069,7 +2076,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:4">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
@@ -2083,7 +2090,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:4">
       <c r="A7" s="1" t="s">
         <v>14</v>
       </c>
@@ -2097,7 +2104,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:4">
       <c r="A8" s="7" t="s">
         <v>1</v>
       </c>
@@ -2111,7 +2118,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:4">
       <c r="A9" s="1" t="s">
         <v>2</v>
       </c>
@@ -2119,7 +2126,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:4">
       <c r="A10" s="1" t="s">
         <v>3</v>
       </c>
@@ -2130,7 +2137,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:4">
       <c r="A11" s="1" t="s">
         <v>42</v>
       </c>
@@ -2144,7 +2151,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:4">
       <c r="A13" t="s">
         <v>37</v>
       </c>
@@ -2153,7 +2160,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:4">
       <c r="A14" t="s">
         <v>38</v>
       </c>
@@ -2163,23 +2170,23 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C10" r:id="rId1" xr:uid="{00000000-0004-0000-0E00-000000000000}"/>
+    <hyperlink ref="C10" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E14"/>
-  <sheetFormatPr defaultColWidth="12.68359375" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.83984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.68359375" customWidth="1"/>
-    <col min="4" max="4" width="26.15625" customWidth="1"/>
+    <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.7109375" customWidth="1"/>
+    <col min="4" max="4" width="26.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:5">
       <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
@@ -2193,7 +2200,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:5">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -2207,7 +2214,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:5">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -2224,7 +2231,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:5">
       <c r="A4" s="2" t="s">
         <v>35</v>
       </c>
@@ -2241,7 +2248,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:5">
       <c r="A5" s="2" t="s">
         <v>16</v>
       </c>
@@ -2255,7 +2262,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:5">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
@@ -2270,7 +2277,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:5">
       <c r="A7" s="1" t="s">
         <v>14</v>
       </c>
@@ -2284,7 +2291,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:5">
       <c r="A8" s="7" t="s">
         <v>1</v>
       </c>
@@ -2298,7 +2305,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:5">
       <c r="A9" s="1" t="s">
         <v>2</v>
       </c>
@@ -2309,7 +2316,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:5">
       <c r="A10" s="1" t="s">
         <v>3</v>
       </c>
@@ -2320,7 +2327,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:5">
       <c r="A11" s="1" t="s">
         <v>42</v>
       </c>
@@ -2334,7 +2341,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:5">
       <c r="A13" t="s">
         <v>37</v>
       </c>
@@ -2343,7 +2350,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:5">
       <c r="A14" t="s">
         <v>38</v>
       </c>
@@ -2359,17 +2366,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D14"/>
-  <sheetFormatPr defaultColWidth="12.68359375" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E14"/>
+  <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.83984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="46.83984375" customWidth="1"/>
-    <col min="4" max="4" width="18.68359375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.7109375" customWidth="1"/>
+    <col min="4" max="4" width="26.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:5">
       <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
@@ -2383,7 +2390,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:5">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -2391,13 +2398,13 @@
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>11</v>
+        <v>102</v>
       </c>
       <c r="D2" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -2407,11 +2414,14 @@
       <c r="C3" t="s">
         <v>18</v>
       </c>
-      <c r="D3" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
       <c r="A4" s="2" t="s">
         <v>35</v>
       </c>
@@ -2424,8 +2434,11 @@
       <c r="D4" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="E4" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
       <c r="A5" s="2" t="s">
         <v>16</v>
       </c>
@@ -2433,13 +2446,10 @@
         <v>60</v>
       </c>
       <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
@@ -2447,41 +2457,41 @@
         <v>7</v>
       </c>
       <c r="C6" t="s">
-        <v>17</v>
+        <v>103</v>
       </c>
       <c r="D6" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:5">
       <c r="A7" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B7" t="s">
         <v>62</v>
       </c>
-      <c r="C7" t="s">
-        <v>51</v>
+      <c r="C7" s="10" t="s">
+        <v>86</v>
       </c>
       <c r="D7" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A8" s="1" t="s">
+    <row r="8" spans="1:5">
+      <c r="A8" s="7" t="s">
         <v>1</v>
       </c>
       <c r="B8" t="s">
         <v>61</v>
       </c>
-      <c r="C8" t="s">
-        <v>13</v>
+      <c r="C8" s="9" t="s">
+        <v>104</v>
       </c>
       <c r="D8" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:5">
       <c r="A9" s="1" t="s">
         <v>2</v>
       </c>
@@ -2492,7 +2502,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:5">
       <c r="A10" s="1" t="s">
         <v>3</v>
       </c>
@@ -2500,10 +2510,10 @@
         <v>6</v>
       </c>
       <c r="C10" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
       <c r="A11" s="1" t="s">
         <v>42</v>
       </c>
@@ -2517,7 +2527,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:5">
       <c r="A13" t="s">
         <v>37</v>
       </c>
@@ -2526,7 +2536,193 @@
         <v>58</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:5">
+      <c r="A14" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14" t="s">
+        <v>63</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>45</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C8" r:id="rId1"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D14"/>
+  <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="46.85546875" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" t="s">
+        <v>62</v>
+      </c>
+      <c r="C7" t="s">
+        <v>51</v>
+      </c>
+      <c r="D7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" t="s">
+        <v>43</v>
+      </c>
+      <c r="D11" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" t="s">
+        <v>37</v>
+      </c>
+      <c r="B13" s="4"/>
+      <c r="C13" s="8" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
       <c r="A14" t="s">
         <v>38</v>
       </c>
@@ -2541,15 +2737,15 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D14"/>
-  <sheetFormatPr defaultColWidth="12.68359375" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.83984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="38.41796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:4">
       <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
@@ -2560,7 +2756,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:4">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -2571,7 +2767,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:4">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -2582,7 +2778,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:4">
       <c r="A4" s="2" t="s">
         <v>35</v>
       </c>
@@ -2593,7 +2789,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:4">
       <c r="A5" s="2" t="s">
         <v>16</v>
       </c>
@@ -2604,7 +2800,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:4">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
@@ -2615,7 +2811,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:4">
       <c r="A7" s="1" t="s">
         <v>14</v>
       </c>
@@ -2626,7 +2822,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:4">
       <c r="A8" s="1" t="s">
         <v>1</v>
       </c>
@@ -2637,7 +2833,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:4">
       <c r="A9" s="1" t="s">
         <v>2</v>
       </c>
@@ -2648,7 +2844,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:4">
       <c r="A10" s="1" t="s">
         <v>3</v>
       </c>
@@ -2659,7 +2855,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:4">
       <c r="A11" s="1" t="s">
         <v>42</v>
       </c>
@@ -2673,7 +2869,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:4">
       <c r="A13" t="s">
         <v>37</v>
       </c>
@@ -2682,7 +2878,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:4">
       <c r="A14" t="s">
         <v>38</v>
       </c>
@@ -2696,14 +2892,14 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J14"/>
-  <sheetFormatPr defaultColWidth="12.68359375" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="15"/>
   <cols>
     <col min="3" max="3" width="21" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:10">
       <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
@@ -2714,7 +2910,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:10">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -2725,7 +2921,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:10">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -2736,7 +2932,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:10">
       <c r="A4" s="2" t="s">
         <v>35</v>
       </c>
@@ -2750,7 +2946,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:10">
       <c r="A5" s="2" t="s">
         <v>16</v>
       </c>
@@ -2761,7 +2957,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:10">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
@@ -2772,7 +2968,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:10" s="5" customFormat="1">
       <c r="A7" s="1" t="s">
         <v>14</v>
       </c>
@@ -2790,7 +2986,7 @@
       <c r="I7" s="6"/>
       <c r="J7" s="6"/>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:10">
       <c r="A8" s="1" t="s">
         <v>1</v>
       </c>
@@ -2801,7 +2997,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:10">
       <c r="A9" s="1" t="s">
         <v>2</v>
       </c>
@@ -2812,7 +3008,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:10">
       <c r="A10" s="1" t="s">
         <v>3</v>
       </c>
@@ -2823,7 +3019,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:10">
       <c r="A11" s="1" t="s">
         <v>42</v>
       </c>
@@ -2831,7 +3027,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:10">
       <c r="A13" t="s">
         <v>37</v>
       </c>
@@ -2840,7 +3036,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:10">
       <c r="A14" t="s">
         <v>38</v>
       </c>
@@ -2854,14 +3050,14 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D14"/>
-  <sheetFormatPr defaultColWidth="12.68359375" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="3" max="3" width="24.26171875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:4">
       <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
@@ -2872,7 +3068,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:4">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -2883,7 +3079,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:4">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -2894,7 +3090,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:4">
       <c r="A4" s="2" t="s">
         <v>35</v>
       </c>
@@ -2908,7 +3104,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:4">
       <c r="A5" s="2" t="s">
         <v>16</v>
       </c>
@@ -2919,7 +3115,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:4">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
@@ -2930,7 +3126,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:4">
       <c r="A7" s="1" t="s">
         <v>14</v>
       </c>
@@ -2941,7 +3137,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:4">
       <c r="A8" s="1" t="s">
         <v>1</v>
       </c>
@@ -2952,7 +3148,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:4">
       <c r="A9" s="1" t="s">
         <v>2</v>
       </c>
@@ -2963,7 +3159,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:4">
       <c r="A10" s="1" t="s">
         <v>3</v>
       </c>
@@ -2974,7 +3170,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:4">
       <c r="A13" t="s">
         <v>37</v>
       </c>
@@ -2983,7 +3179,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:4">
       <c r="A14" t="s">
         <v>38</v>
       </c>
@@ -2997,16 +3193,16 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="12.41796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="39.26171875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="39.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:3">
       <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
@@ -3017,7 +3213,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -3028,7 +3224,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:3">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -3039,7 +3235,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:3">
       <c r="A4" s="2" t="s">
         <v>16</v>
       </c>
@@ -3050,7 +3246,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:3">
       <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
@@ -3061,7 +3257,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:3">
       <c r="A6" s="1" t="s">
         <v>14</v>
       </c>
@@ -3072,7 +3268,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:3">
       <c r="A7" s="1" t="s">
         <v>1</v>
       </c>
@@ -3083,7 +3279,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:3">
       <c r="A8" s="1" t="s">
         <v>2</v>
       </c>
@@ -3094,7 +3290,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:3">
       <c r="A9" s="1" t="s">
         <v>3</v>
       </c>
@@ -3105,7 +3301,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:3">
       <c r="A12" t="s">
         <v>37</v>
       </c>
@@ -3114,7 +3310,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:3">
       <c r="A13" t="s">
         <v>38</v>
       </c>
@@ -3128,16 +3324,16 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="12.41796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="39.26171875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="39.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:3">
       <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
@@ -3148,7 +3344,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -3159,7 +3355,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:3">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -3170,7 +3366,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:3">
       <c r="A4" s="2" t="s">
         <v>16</v>
       </c>
@@ -3181,7 +3377,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:3">
       <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
@@ -3192,7 +3388,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:3">
       <c r="A6" s="1" t="s">
         <v>14</v>
       </c>
@@ -3203,7 +3399,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:3">
       <c r="A7" s="1" t="s">
         <v>1</v>
       </c>
@@ -3214,7 +3410,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:3">
       <c r="A8" s="1" t="s">
         <v>2</v>
       </c>
@@ -3225,7 +3421,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:3">
       <c r="A9" s="1" t="s">
         <v>3</v>
       </c>
@@ -3236,7 +3432,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:3">
       <c r="A12" t="s">
         <v>37</v>
       </c>
@@ -3245,7 +3441,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:3">
       <c r="A13" t="s">
         <v>38</v>
       </c>
@@ -3259,16 +3455,16 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D14"/>
-  <sheetFormatPr defaultColWidth="12.68359375" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="12.41796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.15625" customWidth="1"/>
-    <col min="4" max="4" width="14.26171875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" customWidth="1"/>
+    <col min="4" max="4" width="14.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:4">
       <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
@@ -3282,7 +3478,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:4">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -3293,7 +3489,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:4">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -3304,7 +3500,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:4">
       <c r="A4" s="2" t="s">
         <v>35</v>
       </c>
@@ -3312,7 +3508,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:4">
       <c r="A5" s="2" t="s">
         <v>16</v>
       </c>
@@ -3323,7 +3519,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:4">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
@@ -3334,7 +3530,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:4">
       <c r="A7" s="1" t="s">
         <v>14</v>
       </c>
@@ -3342,7 +3538,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:4">
       <c r="A8" s="7" t="s">
         <v>1</v>
       </c>
@@ -3353,7 +3549,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:4">
       <c r="A9" s="1" t="s">
         <v>2</v>
       </c>
@@ -3361,7 +3557,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:4">
       <c r="A10" s="1" t="s">
         <v>3</v>
       </c>
@@ -3372,7 +3568,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:4">
       <c r="A11" s="1" t="s">
         <v>42</v>
       </c>
@@ -3380,7 +3576,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:4">
       <c r="A13" t="s">
         <v>37</v>
       </c>
@@ -3389,7 +3585,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:4">
       <c r="A14" t="s">
         <v>38</v>
       </c>
@@ -3403,16 +3599,16 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D19"/>
-  <sheetFormatPr defaultColWidth="12.68359375" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="12.41796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.83984375" customWidth="1"/>
-    <col min="4" max="4" width="14.26171875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.85546875" customWidth="1"/>
+    <col min="4" max="4" width="14.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:4">
       <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
@@ -3426,7 +3622,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:4">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -3437,7 +3633,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:4">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -3445,7 +3641,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:4">
       <c r="A4" s="2" t="s">
         <v>35</v>
       </c>
@@ -3456,7 +3652,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:4">
       <c r="A5" s="2" t="s">
         <v>16</v>
       </c>
@@ -3467,7 +3663,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:4">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
@@ -3478,7 +3674,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:4">
       <c r="A7" s="1" t="s">
         <v>14</v>
       </c>
@@ -3486,7 +3682,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:4">
       <c r="A8" s="7" t="s">
         <v>1</v>
       </c>
@@ -3497,7 +3693,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:4">
       <c r="A9" s="1" t="s">
         <v>2</v>
       </c>
@@ -3508,7 +3704,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:4">
       <c r="A10" s="1" t="s">
         <v>3</v>
       </c>
@@ -3516,7 +3712,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:4">
       <c r="A11" s="1" t="s">
         <v>42</v>
       </c>
@@ -3524,7 +3720,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:4">
       <c r="A13" t="s">
         <v>37</v>
       </c>
@@ -3533,7 +3729,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:4">
       <c r="A14" t="s">
         <v>38</v>
       </c>
@@ -3541,12 +3737,12 @@
         <v>45</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:4">
       <c r="A16" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="2:3">
       <c r="B17">
         <v>1</v>
       </c>
@@ -3554,7 +3750,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="2:3">
       <c r="B18">
         <v>2</v>
       </c>
@@ -3562,7 +3758,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="19" spans="2:3">
       <c r="B19">
         <v>3</v>
       </c>

</xml_diff>

<commit_message>
Refactored: Parameter.cs & ParameterExtensions.cs
</commit_message>
<xml_diff>
--- a/Docs/poms.xlsx
+++ b/Docs/poms.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4507"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="23235" windowHeight="12435" activeTab="17"/>
+    <workbookView xWindow="-90" yWindow="-90" windowWidth="23235" windowHeight="12435" activeTab="18"/>
   </bookViews>
   <sheets>
     <sheet name="table" sheetId="1" r:id="rId1"/>
@@ -25,6 +25,7 @@
     <sheet name="partition" sheetId="10" r:id="rId16"/>
     <sheet name="service" sheetId="11" r:id="rId17"/>
     <sheet name="constraint" sheetId="18" r:id="rId18"/>
+    <sheet name="parameter" sheetId="19" r:id="rId19"/>
   </sheets>
   <calcPr calcId="125725"/>
   <extLst>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="688" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="733" uniqueCount="108">
   <si>
     <t xml:space="preserve">id </t>
   </si>
@@ -362,13 +363,57 @@
   </si>
   <si>
     <t>min_value; max_value; column1; column2; ….</t>
+  </si>
+  <si>
+    <r>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>int</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF1A94FF"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF1F377F"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>parameter</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>.Type</t>
+    </r>
+  </si>
+  <si>
+    <t>to {table_id}; to {schema_id}</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="5">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -406,6 +451,30 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Cascadia Mono"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF1A94FF"/>
+      <name val="Cascadia Mono"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF0000FF"/>
+      <name val="Cascadia Mono"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF1F377F"/>
+      <name val="Cascadia Mono"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="5">
@@ -465,7 +534,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -484,6 +553,7 @@
       <alignment shrinkToFit="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -757,7 +827,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2555,6 +2625,193 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E14"/>
+  <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.7109375" customWidth="1"/>
+    <col min="4" max="4" width="26.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="D2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>107</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s">
+        <v>35</v>
+      </c>
+      <c r="D4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E4" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C5">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" t="s">
+        <v>62</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="D7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="D8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" t="s">
+        <v>43</v>
+      </c>
+      <c r="D11" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" t="s">
+        <v>37</v>
+      </c>
+      <c r="B13" s="4"/>
+      <c r="C13" s="8" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14" t="s">
+        <v>63</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>45</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C8" r:id="rId1"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D14"/>

</xml_diff>